<commit_message>
skill tab s5 v4
</commit_message>
<xml_diff>
--- a/docs/2627/misc/DAPR1 skills development.xlsx
+++ b/docs/2627/misc/DAPR1 skills development.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30431"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30502"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{77EA3EEC-57A4-4EC7-A90A-7A999C17A079}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BAC0E3E3-BE11-4B5F-8333-1C5A894077AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -708,13 +708,13 @@
     <t>S5</t>
   </si>
   <si>
-    <t>I can compute appropriate measure(s) of association for a given pair of variables.</t>
+    <t>I can compute measures that summarise how two variables are related</t>
   </si>
   <si>
     <t>V4</t>
   </si>
   <si>
-    <t>I can appropriately plot associations between two variables.</t>
+    <t>I can appropriately plot how two variables are related</t>
   </si>
   <si>
     <t>V3</t>

</xml_diff>